<commit_message>
Change in grouped metrics
</commit_message>
<xml_diff>
--- a/Model/Grouped Metric.xlsx
+++ b/Model/Grouped Metric.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/duonganhtran/Documents/Lecture Notes/Ongoing/31482 Honours Project/Assessment/Assessment 3/AQI Data Analysis - Honours Project/Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{508ABDD0-175A-0D48-9825-71B6218A59CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C5983E-04D4-8944-88FF-2729220908C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1180" windowWidth="27640" windowHeight="16820" xr2:uid="{6AC69E20-3233-7B49-A199-D906AFA5660A}"/>
+    <workbookView xWindow="1080" yWindow="1120" windowWidth="27640" windowHeight="16820" xr2:uid="{6AC69E20-3233-7B49-A199-D906AFA5660A}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Pre" sheetId="1" r:id="rId1"/>
+    <sheet name="During" sheetId="2" r:id="rId2"/>
+    <sheet name="Post" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="15">
   <si>
     <t>pre</t>
   </si>
@@ -88,7 +90,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -144,8 +146,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
@@ -482,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65B33BBF-BC69-274F-86E8-8E5D51D39758}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -538,288 +540,360 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0.84096630999999999</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0.56273764000000004</v>
+      </c>
+      <c r="E3" s="6">
+        <v>37.471482899999998</v>
+      </c>
+      <c r="F3" s="1">
+        <v>784</v>
+      </c>
+      <c r="G3" s="1">
+        <v>261</v>
+      </c>
+      <c r="H3" s="1">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0.86327697999999997</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.60076046000000005</v>
+      </c>
+      <c r="E4" s="6">
+        <v>41.096324500000001</v>
+      </c>
+      <c r="F4" s="1">
+        <v>784</v>
+      </c>
+      <c r="G4" s="1">
+        <v>261</v>
+      </c>
+      <c r="H4" s="1">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.89357657055927298</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.60836501901140605</v>
+      </c>
+      <c r="E5" s="5">
+        <v>40.234474017743899</v>
+      </c>
+      <c r="F5">
+        <v>784</v>
+      </c>
+      <c r="G5">
+        <v>261</v>
+      </c>
+      <c r="H5">
+        <v>263</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FAB6497-D2D3-344A-9E06-148C8C506DCB}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C2" s="3">
         <v>0.90861509746913005</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D2" s="3">
         <v>0.61627906976744096</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E2" s="5">
         <v>33.313953488372</v>
       </c>
-      <c r="F3">
+      <c r="F2">
         <v>255</v>
       </c>
-      <c r="G3">
+      <c r="G2">
         <v>85</v>
       </c>
-      <c r="H3">
+      <c r="H2">
         <v>86</v>
       </c>
     </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0.88921183000000004</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0.60465115999999997</v>
+      </c>
+      <c r="E3" s="6">
+        <v>31.6085271</v>
+      </c>
+      <c r="F3" s="1">
+        <v>255</v>
+      </c>
+      <c r="G3" s="1">
+        <v>85</v>
+      </c>
+      <c r="H3" s="1">
+        <v>86</v>
+      </c>
+    </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0.88921183000000004</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.58139534999999998</v>
+      </c>
+      <c r="E4" s="6">
+        <v>31.6085271</v>
+      </c>
+      <c r="F4" s="1">
+        <v>255</v>
+      </c>
+      <c r="G4" s="1">
+        <v>85</v>
+      </c>
+      <c r="H4" s="1">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.92761258954321502</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.65116279069767402</v>
+      </c>
+      <c r="E5" s="5">
+        <v>33.643410852713103</v>
+      </c>
+      <c r="F5">
+        <v>255</v>
+      </c>
+      <c r="G5">
+        <v>85</v>
+      </c>
+      <c r="H5">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC5C6722-78A1-7342-91BE-3B38C02A5F5F}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C2" s="3">
         <v>0.40443636487610801</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D2" s="3">
         <v>0.156133828996282</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E2" s="5">
         <v>12.267657992565001</v>
       </c>
-      <c r="F4">
+      <c r="F2">
         <v>804</v>
       </c>
-      <c r="G4">
+      <c r="G2">
         <v>268</v>
       </c>
-      <c r="H4">
+      <c r="H2">
         <v>269</v>
       </c>
     </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0.38076425000000003</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0.14498141000000001</v>
+      </c>
+      <c r="E3" s="6">
+        <v>12.0817844</v>
+      </c>
+      <c r="F3" s="1">
+        <v>804</v>
+      </c>
+      <c r="G3" s="1">
+        <v>268</v>
+      </c>
+      <c r="H3" s="1">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0.38076425000000003</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.14498141000000001</v>
+      </c>
+      <c r="E4" s="6">
+        <v>10.966542799999999</v>
+      </c>
+      <c r="F4" s="1">
+        <v>804</v>
+      </c>
+      <c r="G4" s="1">
+        <v>268</v>
+      </c>
+      <c r="H4" s="1">
+        <v>269</v>
+      </c>
+    </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="4">
-        <v>0.84096630999999999</v>
-      </c>
-      <c r="D5" s="4">
-        <v>0.56273764000000004</v>
-      </c>
-      <c r="E5" s="6">
-        <v>37.471482899999998</v>
-      </c>
-      <c r="F5" s="1">
-        <v>784</v>
-      </c>
-      <c r="G5" s="1">
-        <v>261</v>
-      </c>
-      <c r="H5" s="1">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0.88921183000000004</v>
-      </c>
-      <c r="D6" s="4">
-        <v>0.60465115999999997</v>
-      </c>
-      <c r="E6" s="6">
-        <v>31.6085271</v>
-      </c>
-      <c r="F6" s="1">
-        <v>255</v>
-      </c>
-      <c r="G6" s="1">
-        <v>85</v>
-      </c>
-      <c r="H6" s="1">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+      <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="4">
-        <v>0.38076425000000003</v>
-      </c>
-      <c r="D7" s="4">
-        <v>0.14498141000000001</v>
-      </c>
-      <c r="E7" s="6">
-        <v>12.0817844</v>
-      </c>
-      <c r="F7" s="1">
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.456265754425762</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.200743494423791</v>
+      </c>
+      <c r="E5" s="5">
+        <v>17.8438661710037</v>
+      </c>
+      <c r="F5">
         <v>804</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G5">
         <v>268</v>
       </c>
-      <c r="H7" s="1">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="4">
-        <v>0.86327697999999997</v>
-      </c>
-      <c r="D8" s="4">
-        <v>0.60076046000000005</v>
-      </c>
-      <c r="E8" s="6">
-        <v>41.096324500000001</v>
-      </c>
-      <c r="F8" s="1">
-        <v>784</v>
-      </c>
-      <c r="G8" s="1">
-        <v>261</v>
-      </c>
-      <c r="H8" s="1">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="4">
-        <v>0.88921183000000004</v>
-      </c>
-      <c r="D9" s="4">
-        <v>0.58139534999999998</v>
-      </c>
-      <c r="E9" s="6">
-        <v>31.6085271</v>
-      </c>
-      <c r="F9" s="1">
-        <v>255</v>
-      </c>
-      <c r="G9" s="1">
-        <v>85</v>
-      </c>
-      <c r="H9" s="1">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="4">
-        <v>0.38076425000000003</v>
-      </c>
-      <c r="D10" s="4">
-        <v>0.14498141000000001</v>
-      </c>
-      <c r="E10" s="6">
-        <v>10.966542799999999</v>
-      </c>
-      <c r="F10" s="1">
-        <v>804</v>
-      </c>
-      <c r="G10" s="1">
-        <v>268</v>
-      </c>
-      <c r="H10" s="1">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="3">
-        <v>0.89357657055927298</v>
-      </c>
-      <c r="D11" s="3">
-        <v>0.60836501901140605</v>
-      </c>
-      <c r="E11" s="5">
-        <v>40.234474017743899</v>
-      </c>
-      <c r="F11">
-        <v>784</v>
-      </c>
-      <c r="G11">
-        <v>261</v>
-      </c>
-      <c r="H11">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="3">
-        <v>0.92761258954321502</v>
-      </c>
-      <c r="D12" s="3">
-        <v>0.65116279069767402</v>
-      </c>
-      <c r="E12" s="5">
-        <v>33.643410852713103</v>
-      </c>
-      <c r="F12">
-        <v>255</v>
-      </c>
-      <c r="G12">
-        <v>85</v>
-      </c>
-      <c r="H12">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="3">
-        <v>0.456265754425762</v>
-      </c>
-      <c r="D13" s="3">
-        <v>0.200743494423791</v>
-      </c>
-      <c r="E13" s="5">
-        <v>17.8438661710037</v>
-      </c>
-      <c r="F13">
-        <v>804</v>
-      </c>
-      <c r="G13">
-        <v>268</v>
-      </c>
-      <c r="H13">
+      <c r="H5">
         <v>269</v>
       </c>
     </row>

</xml_diff>